<commit_message>
Update robot control parameters and add new class resources
- Adjusted the minimum and maximum values for the right arm in `Mega.ino` to improve control accuracy.
- Updated the `Esp32.ino` file to reflect changes in the right arm's limits and positions.
- Added new classes and resources for "Clase 1 Español 5to" and "Clase 2 Estudios Sociales," including Python scripts, configuration files, and PDFs.
- Enhanced the sequence JSON files to optimize robot movements and ensure better performance.
- Updated metadata and configuration files to include new classes and their respective details.
</commit_message>
<xml_diff>
--- a/Excels.xlsx
+++ b/Excels.xlsx
@@ -1,10 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" mc:Ignorable="x15">
-  <fileVersion appName="xl" lastEdited="6" lowestEdited="6" rupBuild="14420"/>
-  <workbookPr defaultThemeVersion="164011"/>
+<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="6" rupBuild="29231"/>
+  <workbookPr/>
+  <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
+    <mc:Choice Requires="x15">
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\josue\Desktop\RobotAtlas\"/>
+    </mc:Choice>
+  </mc:AlternateContent>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{FABEAF58-72C8-44E6-B272-DCC71CDB6DCD}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="0" yWindow="0" windowWidth="22260" windowHeight="12645"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="24240" windowHeight="13020" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
@@ -18,10 +24,77 @@
 </workbook>
 </file>
 
+<file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="18" uniqueCount="18">
+  <si>
+    <t>Comando</t>
+  </si>
+  <si>
+    <t>Parámetros</t>
+  </si>
+  <si>
+    <t>Función</t>
+  </si>
+  <si>
+    <t>BRAZOS</t>
+  </si>
+  <si>
+    <t>BI, BD, FI, FD, HI, HD, PD</t>
+  </si>
+  <si>
+    <t>Posicionar brazos</t>
+  </si>
+  <si>
+    <t>MANO</t>
+  </si>
+  <si>
+    <t>M, GESTO o DEDO+ANG</t>
+  </si>
+  <si>
+    <t>Gestos o dedos individuales</t>
+  </si>
+  <si>
+    <t>MUÑECA</t>
+  </si>
+  <si>
+    <t>mano, ángulo</t>
+  </si>
+  <si>
+    <t>Rotar muñeca</t>
+  </si>
+  <si>
+    <t>CUELLO</t>
+  </si>
+  <si>
+    <t>L, I, S</t>
+  </si>
+  <si>
+    <t>Mover cuello</t>
+  </si>
+  <si>
+    <t>HABLAR</t>
+  </si>
+  <si>
+    <t>texto</t>
+  </si>
+  <si>
+    <t>Sintetizar voz</t>
+  </si>
+</sst>
+</file>
+
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
-<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" mc:Ignorable="x14ac x16r2">
-  <fonts count="1" x14ac:knownFonts="1">
+<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
+  <fonts count="2" x14ac:knownFonts="1">
     <font>
+      <sz val="11"/>
+      <color theme="1"/>
+      <name val="Calibri"/>
+      <family val="2"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <b/>
       <sz val="11"/>
       <color theme="1"/>
       <name val="Calibri"/>
@@ -37,7 +110,7 @@
       <patternFill patternType="gray125"/>
     </fill>
   </fills>
-  <borders count="1">
+  <borders count="2">
     <border>
       <left/>
       <right/>
@@ -45,12 +118,36 @@
       <bottom/>
       <diagonal/>
     </border>
+    <border>
+      <left style="thin">
+        <color indexed="64"/>
+      </left>
+      <right style="thin">
+        <color indexed="64"/>
+      </right>
+      <top style="thin">
+        <color indexed="64"/>
+      </top>
+      <bottom style="thin">
+        <color indexed="64"/>
+      </bottom>
+      <diagonal/>
+    </border>
   </borders>
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="1">
+  <cellXfs count="4">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center" wrapText="1"/>
+    </xf>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -330,10 +427,82 @@
 </file>
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
-  <dimension ref="A1"/>
-  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
-  <sheetData/>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
+  <dimension ref="D9:F14"/>
+  <sheetFormatPr baseColWidth="10" defaultColWidth="9.140625" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <cols>
+    <col min="5" max="5" width="26.28515625" customWidth="1"/>
+    <col min="6" max="6" width="30.28515625" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="9" spans="4:6" ht="30" x14ac:dyDescent="0.25">
+      <c r="D9" s="1" t="s">
+        <v>0</v>
+      </c>
+      <c r="E9" s="1" t="s">
+        <v>1</v>
+      </c>
+      <c r="F9" s="1" t="s">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="10" spans="4:6" ht="33.75" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="D10" s="2" t="s">
+        <v>3</v>
+      </c>
+      <c r="E10" s="3" t="s">
+        <v>4</v>
+      </c>
+      <c r="F10" s="3" t="s">
+        <v>5</v>
+      </c>
+    </row>
+    <row r="11" spans="4:6" ht="21.75" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="D11" s="2" t="s">
+        <v>6</v>
+      </c>
+      <c r="E11" s="3" t="s">
+        <v>7</v>
+      </c>
+      <c r="F11" s="3" t="s">
+        <v>8</v>
+      </c>
+    </row>
+    <row r="12" spans="4:6" ht="30" x14ac:dyDescent="0.25">
+      <c r="D12" s="2" t="s">
+        <v>9</v>
+      </c>
+      <c r="E12" s="3" t="s">
+        <v>10</v>
+      </c>
+      <c r="F12" s="3" t="s">
+        <v>11</v>
+      </c>
+    </row>
+    <row r="13" spans="4:6" ht="30" x14ac:dyDescent="0.25">
+      <c r="D13" s="2" t="s">
+        <v>12</v>
+      </c>
+      <c r="E13" s="3" t="s">
+        <v>13</v>
+      </c>
+      <c r="F13" s="3" t="s">
+        <v>14</v>
+      </c>
+    </row>
+    <row r="14" spans="4:6" ht="30" x14ac:dyDescent="0.25">
+      <c r="D14" s="2" t="s">
+        <v>15</v>
+      </c>
+      <c r="E14" s="3" t="s">
+        <v>16</v>
+      </c>
+      <c r="F14" s="3" t="s">
+        <v>17</v>
+      </c>
+    </row>
+  </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+  <pageSetup paperSize="9" orientation="portrait" r:id="rId1"/>
 </worksheet>
 </file>
</xml_diff>